<commit_message>
Added storeTests and petTests
</commit_message>
<xml_diff>
--- a/testData/userData.xlsx
+++ b/testData/userData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="153222"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14796" windowHeight="4128"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14796" windowHeight="4308"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -430,7 +430,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G13"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="7" max="7" width="11" bestFit="1" customWidth="1"/>
@@ -528,6 +528,21 @@
         <v>1234567890</v>
       </c>
     </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="3"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3"/>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3"/>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E2" r:id="rId1"/>

</xml_diff>